<commit_message>
Arregla el generador del modelo, que no funcionaba fuera de esta máquina
La revisión destapó que el script publicado llevaba dentro la ruta
absoluta de una carpeta temporal de sesión. Nadie más podía ejecutarlo, y
esta misma máquina dejó de poder en cuanto el temporal se limpió. Ahora
openpyxl se declara como extra del proyecto y el script lo importa
normalmente, con un mensaje que dice qué instalar si falta.

Además, dos celdas de la calculadora salían como #NAME? en Excel: las
etiquetas empezaban por "=" y Excel las tomaba por fórmulas. Y seis avisos
de ruff por imports duplicados que el CI habría rechazado.

Comprobado que el generador reproduce el libro publicado sin una sola
celda de diferencia, y que los valores que Excel calcula coinciden con el
cálculo hecho aparte.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Noesis-Modelo-Economico.xlsx
+++ b/docs/Noesis-Modelo-Economico.xlsx
@@ -754,11 +754,6 @@
           <t>Catalogo adoptado</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -890,11 +885,6 @@
           <t>Resultado por plan (modelo Noesis)</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1058,11 +1048,6 @@
           <t>Punto de equilibrio</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1206,28 +1191,9 @@
           <t>Ninguna cifra de este libro es un resultado observado. Son supuestos de planificacion fechados que el piloto debe recalibrar. El opex fijo, los sueldos, el reparto societario y el CAC no constan en el repositorio: estan en Datos_Pendientes sin rellenar.</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-    </row>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A10:F10"/>
@@ -5393,7 +5359,7 @@
         </is>
       </c>
       <c r="B6" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="15">
         <f>Supuestos!B7</f>
@@ -5415,7 +5381,7 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C7" s="15">
         <f>Supuestos!C7</f>
@@ -5437,7 +5403,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8" s="15">
         <f>Supuestos!D7</f>
@@ -6025,9 +5991,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16">
-        <f> Margen bruto</f>
-        <v/>
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>MARGEN BRUTO</t>
+        </is>
       </c>
       <c r="B39" s="23">
         <f>B37+B38</f>
@@ -6084,9 +6051,10 @@
       </c>
     </row>
     <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="16">
-        <f> RESULTADO</f>
-        <v/>
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>RESULTADO DEL MES</t>
+        </is>
       </c>
       <c r="B42" s="26">
         <f>B39+B40+B41</f>

</xml_diff>